<commit_message>
updated to reflect table in 3a
</commit_message>
<xml_diff>
--- a/week-09/NorthwindTablesAndColumns.xlsx
+++ b/week-09/NorthwindTablesAndColumns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Longley\Documents\DataAnalytics\week-09\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E87B88-D66A-45A7-B03C-F3E0509857EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65D7AC21-7FA9-4E6A-A2DA-6B7F0324A3C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="10500" windowWidth="19200" windowHeight="10500" xr2:uid="{901F5D27-877F-4C94-89AE-9A9B6ECE5CB6}"/>
+    <workbookView xWindow="3465" yWindow="5520" windowWidth="15600" windowHeight="10995" xr2:uid="{901F5D27-877F-4C94-89AE-9A9B6ECE5CB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Northwind Columns" sheetId="1" r:id="rId1"/>
@@ -875,7 +875,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -898,7 +898,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -927,7 +927,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -947,7 +947,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -967,7 +967,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -990,7 +990,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>60</v>
       </c>
       <c r="H8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
@@ -1056,10 +1056,10 @@
         <v>60</v>
       </c>
       <c r="H9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
@@ -1169,7 +1169,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
@@ -1238,7 +1238,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>40</v>
       </c>
       <c r="H18" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
@@ -1298,7 +1298,7 @@
         <v>20</v>
       </c>
       <c r="H19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
@@ -1318,7 +1318,7 @@
         <v>60</v>
       </c>
       <c r="H20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
@@ -1338,10 +1338,10 @@
         <v>50</v>
       </c>
       <c r="H21" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>27</v>
       </c>
@@ -1405,7 +1405,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>27</v>
       </c>
@@ -1425,7 +1425,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>27</v>
       </c>
@@ -1454,7 +1454,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>27</v>
       </c>
@@ -1483,7 +1483,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
@@ -1544,7 +1544,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>27</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>27</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>27</v>
       </c>
@@ -1624,7 +1624,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>27</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>27</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>42</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>42</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>44</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>44</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>44</v>
       </c>
@@ -1832,7 +1832,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>44</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>53</v>
       </c>
@@ -1887,7 +1887,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>53</v>
       </c>
@@ -1910,7 +1910,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>53</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>53</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>53</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>53</v>
       </c>
@@ -2029,7 +2029,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>53</v>
       </c>
@@ -2061,7 +2061,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>53</v>
       </c>
@@ -2107,10 +2107,10 @@
         <v>80</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>53</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>53</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>53</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>53</v>
       </c>
@@ -2220,7 +2220,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>65</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>65</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>65</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>65</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>65</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>65</v>
       </c>
@@ -2411,7 +2411,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>65</v>
       </c>
@@ -2443,7 +2443,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>65</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>65</v>
       </c>
@@ -2521,10 +2521,10 @@
         <v>1</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>22</v>
       </c>
@@ -2564,10 +2564,10 @@
         <v>100</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>76</v>
       </c>
@@ -2590,7 +2590,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>76</v>
       </c>
@@ -2619,7 +2619,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>76</v>
       </c>
@@ -2639,7 +2639,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>78</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>78</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>60</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
@@ -2728,10 +2728,10 @@
         <v>60</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="75" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>78</v>
       </c>
@@ -2751,7 +2751,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>78</v>
       </c>
@@ -2780,7 +2780,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>78</v>
       </c>
@@ -2809,7 +2809,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>78</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="80" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
@@ -2890,7 +2890,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>78</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>78</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>80</v>
       </c>
@@ -2970,10 +2970,10 @@
         <v>100</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>80</v>
       </c>
@@ -3000,7 +3000,7 @@
   <autoFilter ref="A1:N85" xr:uid="{A6B56A5E-AA28-4DB9-BAE3-51DE131C631E}">
     <filterColumn colId="7">
       <filters>
-        <filter val="keep."/>
+        <filter val="no"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -3009,6 +3009,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA5D0A6329BB324E86983B32928CFC2E" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d7eac4bce3bbb09c82bd908806be82e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xmlns:ns3="ced60a7f-99b1-48d2-b555-34851c8026ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb51570e5b7cb8bd524bc2df5324d4a3" ns2:_="" ns3:_="">
     <xsd:import namespace="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
@@ -3249,25 +3268,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3278,6 +3278,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB560F9-4CC1-4243-8F16-7FDC2CD703FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
+    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA285021-94D7-4152-B2E7-B2D9504C2DBD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3296,17 +3307,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB560F9-4CC1-4243-8F16-7FDC2CD703FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
-    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0257D61C-6042-483B-9C34-3DE0D82CB154}">
   <ds:schemaRefs>

</xml_diff>